<commit_message>
fix: populate all 289 consumables
populate all 289 consumables, 60 resistance enchants, and 339 normal
sealbooks
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/enchants.xlsx
+++ b/mod_project/data_tables/enchants.xlsx
@@ -2871,12 +2871,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Fire resistance UP</t>
+          <t>Fire Res +20</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2903,12 +2903,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Fire resistance MiniUP</t>
+          <t>Fire Res +10</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2935,12 +2935,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Fire resistance DOWN</t>
+          <t>Fire Res -20</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2967,12 +2967,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Water resistance UP</t>
+          <t>Water Res +20</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -2999,12 +2999,12 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Water resistance MiniUP</t>
+          <t>Water Res +10</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3031,12 +3031,12 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Water resistance DOWN</t>
+          <t>Water Res -20</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3063,12 +3063,12 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Wind resistance UP</t>
+          <t>Wind Res +20</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3095,12 +3095,12 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Wind resistance MiniUP</t>
+          <t>Wind Res +10</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3127,12 +3127,12 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Wind resistance DOWN</t>
+          <t>Wind Res -20</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3159,12 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Earth resistance UP</t>
+          <t>Earth Res +20</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3191,12 +3191,12 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Earth resistance MiniUP</t>
+          <t>Earth Res +10</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3223,12 +3223,12 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Earth resistance DOWN</t>
+          <t>Earth Res -20</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3255,12 +3255,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Lightning resistance UP</t>
+          <t>Lightning Res +20</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3287,12 +3287,12 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Lightning resistance MiniUP</t>
+          <t>Lightning Res +10</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3319,12 +3319,12 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Lightning resistance DOWN</t>
+          <t>Lightning Res -20</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3351,12 +3351,12 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Elemental resistance GrandUP</t>
+          <t>All Elem Res +50</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3383,12 +3383,12 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Elemental resistance UP</t>
+          <t>All Elem Res +15</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3415,12 +3415,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Elemental resistance MiniUP</t>
+          <t>All Elem Res +7</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3447,12 +3447,12 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Elemental resistance DOWN</t>
+          <t>All Elem Res -15</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3479,12 +3479,12 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Slash resistance UP</t>
+          <t>Slash Res +20</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3511,12 +3511,12 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Slash resistance MiniUP</t>
+          <t>Slash Res +10</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3543,12 +3543,12 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Slash resistance DOWN</t>
+          <t>Slash Res -20</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3575,12 +3575,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Stab resistance UP</t>
+          <t>Stab Res +20</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3607,12 +3607,12 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Stab resistance MiniUP</t>
+          <t>Stab Res +10</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3639,12 +3639,12 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Stab resistance DOWN</t>
+          <t>Stab Res -20</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3671,12 +3671,12 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Bash resistance UP</t>
+          <t>Bash Res +20</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3703,12 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Bash resistance MiniUP</t>
+          <t>Bash Res +10</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3735,12 +3735,12 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Bash resistance DOWN</t>
+          <t>Bash Res -20</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3767,12 +3767,12 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Physical resistance GrandUP</t>
+          <t>All Phys Res +50</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3799,12 +3799,12 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>Physical resistance UP</t>
+          <t>All Phys Res +15</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3831,12 +3831,12 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>Physical resistance MiniUP</t>
+          <t>All Phys Res +7</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -3863,12 +3863,12 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Physical resistance DOWN</t>
+          <t>All Phys Res -15</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8535,12 +8535,12 @@
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>Fire resistance MegaUP</t>
+          <t>Fire Res +30</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8567,12 +8567,12 @@
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>Fire resistance GrandUP</t>
+          <t>Fire Res +50</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8599,12 +8599,12 @@
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>Fire resistance GrandDOWN</t>
+          <t>Fire Res -40</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8631,12 +8631,12 @@
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>Water resistance MegaUP</t>
+          <t>Water Res +30</t>
         </is>
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8663,12 +8663,12 @@
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>Water resistance GrandUP</t>
+          <t>Water Res +50</t>
         </is>
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8695,12 +8695,12 @@
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>Water resistance GrandDOWN</t>
+          <t>Water Res -40</t>
         </is>
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8727,12 +8727,12 @@
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>Wind resistance MegaUP</t>
+          <t>Wind Res +30</t>
         </is>
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8759,12 +8759,12 @@
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>Wind resistance GrandUP</t>
+          <t>Wind Res +50</t>
         </is>
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8791,12 +8791,12 @@
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>Wind resistance GrandDOWN</t>
+          <t>Wind Res -40</t>
         </is>
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8823,12 +8823,12 @@
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>Earth resistance MegaUP</t>
+          <t>Earth Res +30</t>
         </is>
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8855,12 +8855,12 @@
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>Earth resistance GrandUP</t>
+          <t>Earth Res +50</t>
         </is>
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8887,12 +8887,12 @@
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>Earth resistance GrandDOWN</t>
+          <t>Earth Res -40</t>
         </is>
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8919,12 +8919,12 @@
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>Lightning resistance MegaUP</t>
+          <t>Lightning Res +30</t>
         </is>
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8951,12 +8951,12 @@
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>Lightning resistance GrandUP</t>
+          <t>Lightning Res +50</t>
         </is>
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8983,12 +8983,12 @@
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>Lightning resistance GrandDOWN</t>
+          <t>Lightning Res -40</t>
         </is>
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9015,12 +9015,12 @@
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>Elemental resistance MegaUP</t>
+          <t>All Elem Res +30</t>
         </is>
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9047,12 +9047,12 @@
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>Elemental resistance GrandDOWN</t>
+          <t>All Elem Res -30</t>
         </is>
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9079,12 +9079,12 @@
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>Slash resistance MegaUP</t>
+          <t>Slash Res +30</t>
         </is>
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9111,12 +9111,12 @@
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>Slash resistance GrandUP</t>
+          <t>Slash Res +50</t>
         </is>
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9143,12 +9143,12 @@
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>Slash resistance GrandDOWN</t>
+          <t>Slash Res -40</t>
         </is>
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9175,12 +9175,12 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>Stab resistance MegaUP</t>
+          <t>Stab Res +30</t>
         </is>
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9207,12 +9207,12 @@
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>Stab resistance GrandUP</t>
+          <t>Stab Res +50</t>
         </is>
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9239,12 +9239,12 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Stab resistance GrandDOWN</t>
+          <t>Stab Res -40</t>
         </is>
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9271,12 +9271,12 @@
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>Bash resistance MegaUP</t>
+          <t>Bash Res +30</t>
         </is>
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9303,12 +9303,12 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Bash resistance GrandUP</t>
+          <t>Bash Res +50</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9335,12 +9335,12 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Bash resistance GrandDOWN</t>
+          <t>Bash Res -40</t>
         </is>
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9367,12 +9367,12 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Physical resistance MegaUP</t>
+          <t>All Phys Res +30</t>
         </is>
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -9399,12 +9399,12 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Physical resistance GrandDOWN</t>
+          <t>All Phys Res -30</t>
         </is>
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: upgrade 52 equipment enchants including HP/TP regen on Nurse Cap
upgrade 52 equipment enchants including HP/TP regen on Nurse Cap and
race slayers
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/enchants.xlsx
+++ b/mod_project/data_tables/enchants.xlsx
@@ -4535,7 +4535,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>HP Regen +50/turn</t>
+          <t>HP Regen +4%/turn</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -4567,12 +4567,12 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>Slight HP recovery every turn</t>
+          <t>HP Regen +2%/turn</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>TP Regen +10/turn</t>
+          <t>TP Regen +4/turn</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -4631,12 +4631,12 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Slight TP recovery every turn</t>
+          <t>TP Regen +2/turn</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4663,12 +4663,12 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>Large HP recovery every turn</t>
+          <t>HP Regen +8%/turn</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4695,12 +4695,12 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Large TP recovery every turn</t>
+          <t>TP Regen +6/turn</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4983,12 +4983,12 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Normal attacks absorb lots of HP</t>
+          <t>Normal attacks: 50% HP Drain</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5015,12 +5015,12 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Normal attacks absorb HP</t>
+          <t>Normal attacks: 20% HP Drain</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5047,12 +5047,12 @@
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>Normal attacks absorb lots of TP</t>
+          <t>Normal attacks: 20% TP Drain</t>
         </is>
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5079,12 +5079,12 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Normal attacks absorb TP</t>
+          <t>Normal attacks: 10% TP Drain</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5143,12 +5143,12 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons GrandUP</t>
+          <t>Physical ATK vs. Demons +50%</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5175,12 +5175,12 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons UP</t>
+          <t>Physical ATK vs. Demons +20%</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5207,12 +5207,12 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions GrandUP</t>
+          <t>Physical ATK vs. Apparitions +50%</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5239,12 +5239,12 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions UP</t>
+          <t>Physical ATK vs. Apparitions +20%</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5271,12 +5271,12 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Magic Beings GrandUP</t>
+          <t>Physical ATK vs. Magic Beings +50%</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5303,12 +5303,12 @@
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>Physical attack vs. Magic Beings UP</t>
+          <t>Physical ATK vs. Magic Beings +20%</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans MegaUP</t>
+          <t>Physical ATK vs. Humans +100%</t>
         </is>
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5367,12 +5367,12 @@
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans GrandUP</t>
+          <t>Physical ATK vs. Humans +50%</t>
         </is>
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5399,12 +5399,12 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans UP</t>
+          <t>Physical ATK vs. Humans +20%</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5431,12 +5431,12 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead GrandUP</t>
+          <t>Physical ATK vs. Undead +50%</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5463,12 +5463,12 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead UP</t>
+          <t>Physical ATK vs. Undead +20%</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5495,12 +5495,12 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons GrandUP</t>
+          <t>Physical ATK vs. Dragons +50%</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5527,12 +5527,12 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons UP</t>
+          <t>Physical ATK vs. Dragons +20%</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5559,12 +5559,12 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts GrandUP</t>
+          <t>Physical ATK vs. Beasts +50%</t>
         </is>
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5591,12 +5591,12 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts UP</t>
+          <t>Physical ATK vs. Beasts +20%</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5623,12 +5623,12 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>Physical attack vs. Fruit MegaUP</t>
+          <t>Physical ATK vs. Fruit +100%</t>
         </is>
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5655,12 +5655,12 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>Physical attack vs. Fruit GrandUP</t>
+          <t>Physical ATK vs. Fruit +50%</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5815,12 +5815,12 @@
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Physical attack vs. Felines MegaUP</t>
+          <t>Physical ATK vs. Felines +100%</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5943,12 +5943,12 @@
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons MegaUP</t>
+          <t>Physical ATK vs. Demons +100%</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5975,12 +5975,12 @@
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions MegaUP</t>
+          <t>Physical ATK vs. Apparitions +100%</t>
         </is>
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6007,12 +6007,12 @@
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Magic Beings MegaUP</t>
+          <t>Physical ATK vs. Magic Beings +100%</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6039,12 +6039,12 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead MegaUP</t>
+          <t>Physical ATK vs. Undead +100%</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6071,12 +6071,12 @@
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons MegaUP</t>
+          <t>Physical ATK vs. Dragons +100%</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6103,12 +6103,12 @@
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts MegaUP</t>
+          <t>Physical ATK vs. Beasts +100%</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6135,12 +6135,12 @@
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Sea Creatures MegaUP</t>
+          <t>Physical ATK vs. Sea Creatures +100%</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6167,12 +6167,12 @@
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>Slightly reduce encounter rate</t>
+          <t>Encounter Rate -25%</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6199,12 +6199,12 @@
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>Greatly reduce encounter rate</t>
+          <t>Encounter Rate -50%</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6231,12 +6231,12 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>Slightly increase encounter rate</t>
+          <t>Encounter Rate +25%</t>
         </is>
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6263,12 +6263,12 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>Greatly increase encounter rate</t>
+          <t>Encounter Rate +50%</t>
         </is>
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7127,12 +7127,12 @@
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>TP Cost for techniques DOWN</t>
+          <t>Technique TP Cost -10%</t>
         </is>
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7159,12 +7159,12 @@
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>TP Cost for techniques MegaDOWN</t>
+          <t>Technique TP Cost -25%</t>
         </is>
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7191,12 +7191,12 @@
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>TP Cost for spells DOWN</t>
+          <t>Spell TP Cost -10%</t>
         </is>
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7223,12 +7223,12 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>TP Cost for spells MegaDOWN</t>
+          <t>Spell TP Cost -25%</t>
         </is>
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7415,12 +7415,12 @@
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>HP recovers while defending</t>
+          <t>Defending HP Regen +10%</t>
         </is>
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7543,12 +7543,12 @@
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>Damage of joint skills UP</t>
+          <t>Joint Skill Damage +25%</t>
         </is>
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7575,12 +7575,12 @@
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>Escape probability UP</t>
+          <t>Escape Chance +25%</t>
         </is>
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7959,12 +7959,12 @@
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>Equipment drop rate UP</t>
+          <t>Equipment Drop Rate +25%</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7991,12 +7991,12 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Damage to enemies with status ailments UP</t>
+          <t>Damage vs. Ailment Foes +25%</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8055,12 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Joint skill damage MegaUP</t>
+          <t>Joint Skill Damage +50%</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8119,12 +8119,12 @@
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>TP recovers slightly while defending</t>
+          <t>Defending TP Regen +10</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8215,12 +8215,12 @@
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>Increase Mercenary Buddy stats by 10%</t>
+          <t>Mercenary Buddy Stats +10%</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8279,12 +8279,12 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Increase Mercenary Buddy stats by 30</t>
+          <t>Mercenary Buddy Stats +30</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete Crown enchant descriptions for Grand Sealbooks
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/enchants.xlsx
+++ b/mod_project/data_tables/enchants.xlsx
@@ -6327,12 +6327,12 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>Recover 3 TP every 10 steps</t>
+          <t>Recover 3 TP / 10 steps</t>
         </is>
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6359,12 +6359,12 @@
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>Attack vs. high lvl enemies UP</t>
+          <t>ATK vs. Higher-Level Foes +25%</t>
         </is>
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6391,12 +6391,12 @@
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>Attack vs. low lvl enemies UP</t>
+          <t>ATK vs. Lower-Level Foes +25%</t>
         </is>
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6423,12 +6423,12 @@
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>Front line ATK 8% UP</t>
+          <t>Front Row ATK +8%</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6455,12 +6455,12 @@
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>Front line ATK + DEF 4% UP</t>
+          <t>Front Row ATK/DEF +4%</t>
         </is>
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6487,12 +6487,12 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>Back line INT 8% UP</t>
+          <t>Back Row INT +8%</t>
         </is>
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6519,12 +6519,12 @@
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>Back line INT + RES 4% UP</t>
+          <t>Back Row INT/RES +4%</t>
         </is>
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7447,12 +7447,12 @@
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>Higher lvl equipment from treasure boxes</t>
+          <t>Treasure Chest Item Level +1</t>
         </is>
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7479,12 +7479,12 @@
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>Higher chance of shop encounters</t>
+          <t>Wandering Shop Encounter Rate +50%</t>
         </is>
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7511,12 +7511,12 @@
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>Damage from non-gas traps 90% DOWN</t>
+          <t>Non-Gas Trap Damage -90%</t>
         </is>
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7607,12 +7607,12 @@
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>A-rank speed when no weapon is equipped</t>
+          <t>Unarmed Action Speed: A-Rank</t>
         </is>
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7639,12 +7639,12 @@
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>Class weapon modifier 2% UP</t>
+          <t>Class Weapon Modifier +2%</t>
         </is>
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7671,12 +7671,12 @@
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Rate of status ailments dissipation UP</t>
+          <t>Ailment Natural Recovery Rate +50%</t>
         </is>
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7703,12 +7703,12 @@
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>Pep decrease rate DOWN</t>
+          <t>Pep Decrease Rate -50%</t>
         </is>
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7735,12 +7735,12 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>The smaller your party, the higher your damage</t>
+          <t>Damage +100%/empty party slot</t>
         </is>
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7831,12 +7831,12 @@
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>Gain more EXP from higher-level enemies</t>
+          <t>Higher-Level Enemy EXP +50%</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7863,12 +7863,12 @@
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>When max HP, damage inflicted 10% UP</t>
+          <t>Damage at Max HP +10%</t>
         </is>
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7895,12 +7895,12 @@
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>Reduce damage penalty for missed spells</t>
+          <t>Missed Spell Damage Penalty -50%</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8023,12 +8023,12 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Back line DEX + AGI 2% UP</t>
+          <t>Back Row DEX/AGI +2%</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8087,12 +8087,12 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Increase Mimic appearance rate in chests</t>
+          <t>Chest Mimic Appearance Rate UP</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8151,12 +8151,12 @@
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>Unique skill level +1</t>
+          <t>Unique Skill Level +1</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8183,12 +8183,12 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>Food likes and dislikes intensify</t>
+          <t>Food Affinity Bonus/Penalty x2</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8247,12 +8247,12 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>May rarely recover all HP when turn starts</t>
+          <t>Turn Start Full HP Recovery (10%)</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8311,12 +8311,12 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>Magic incantations go very fast... sometimes</t>
+          <t>Fast Spell Cast (Instant Cast chance)</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete overhaul of enchants
complete overhaul of enchants, monster attacks, and grand seal crowns
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/enchants.xlsx
+++ b/mod_project/data_tables/enchants.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,32 +429,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>File_Name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Vanilla_Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Prefix</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Suffix</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Modded_Name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -4727,12 +4739,12 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict poison</t>
+          <t>Normal attacks: Poison chance (20%)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4759,12 +4771,12 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict sleep</t>
+          <t>Normal attacks: Sleep chance (20%)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4791,12 +4803,12 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict silence</t>
+          <t>Normal attacks: Silence chance (20%)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4823,12 +4835,12 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict freeze</t>
+          <t>Normal attacks: Freeze chance (20%)</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4855,12 +4867,12 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict paralysis</t>
+          <t>Normal attacks: Paralysis chance (20%)</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4887,12 +4899,12 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict stun</t>
+          <t>Normal attacks: Stun chance (20%)</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4919,12 +4931,12 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict petrification</t>
+          <t>Normal attacks: Petrify chance (15%)</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -4951,12 +4963,12 @@
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>Normal attacks may instakill</t>
+          <t>Normal attacks: Instakill chance (15%)</t>
         </is>
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5111,12 +5123,12 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>Normal attacks may inflict slow</t>
+          <t>Normal attacks: Slow chance (15%)</t>
         </is>
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -5847,12 +5859,12 @@
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>Normal attacks will probably instakill</t>
+          <t>Normal attacks: High Instakill chance (50%)</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6551,12 +6563,12 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>Damage from Demons 5% DOWN</t>
+          <t>Damage from Demons -5%</t>
         </is>
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6583,12 +6595,12 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>Damage from Demons 10% DOWN</t>
+          <t>Damage from Demons -10%</t>
         </is>
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6615,12 +6627,12 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>Damage from Apparitions 5% DOWN</t>
+          <t>Damage from Apparitions -5%</t>
         </is>
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6647,12 +6659,12 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>Damage from Apparitions 10% DOWN</t>
+          <t>Damage from Apparitions -10%</t>
         </is>
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6679,12 +6691,12 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>Damage from Magic Beings 5% DOWN</t>
+          <t>Damage from Magic Beings -5%</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6711,12 +6723,12 @@
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>Damage from Magic Beings 10% DOWN</t>
+          <t>Damage from Magic Beings -10%</t>
         </is>
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6743,12 +6755,12 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>Damage from Humans 5% DOWN</t>
+          <t>Damage from Humans -5%</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6775,12 +6787,12 @@
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>Damage from Humans 10% DOWN</t>
+          <t>Damage from Humans -10%</t>
         </is>
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6807,12 +6819,12 @@
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>Damage from Undead 5% DOWN</t>
+          <t>Damage from Undead -5%</t>
         </is>
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6839,12 +6851,12 @@
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>Damage from Undead 10% DOWN</t>
+          <t>Damage from Undead -10%</t>
         </is>
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6871,12 +6883,12 @@
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>Damage from Dragons 5% DOWN</t>
+          <t>Damage from Dragons -5%</t>
         </is>
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6903,12 +6915,12 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>Damage from Dragons 10% DOWN</t>
+          <t>Damage from Dragons -10%</t>
         </is>
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6935,12 +6947,12 @@
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>Damage from Beasts 5% DOWN</t>
+          <t>Damage from Beasts -5%</t>
         </is>
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6967,12 +6979,12 @@
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>Damage from Beasts 10% DOWN</t>
+          <t>Damage from Beasts -10%</t>
         </is>
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -6999,12 +7011,12 @@
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>Damage from Fruit 5% DOWN</t>
+          <t>Damage from Fruit -5%</t>
         </is>
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7031,12 +7043,12 @@
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>Damage from Fruit 10% DOWN</t>
+          <t>Damage from Fruit -10%</t>
         </is>
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7063,12 +7075,12 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>Damage from Therians 5% DOWN</t>
+          <t>Damage from Therians -5%</t>
         </is>
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7095,12 +7107,12 @@
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>Damage from Therians 10% DOWN</t>
+          <t>Damage from Therians -10%</t>
         </is>
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7255,12 +7267,12 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Fire attack for both sides UP</t>
+          <t>Fire Attack for all allies &amp; foes +25%</t>
         </is>
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7287,12 +7299,12 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Water attack for both sides UP</t>
+          <t>Water Attack for all allies &amp; foes +25%</t>
         </is>
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7319,12 +7331,12 @@
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>Wind attack for both sides UP</t>
+          <t>Wind Attack for all allies &amp; foes +25%</t>
         </is>
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7351,12 +7363,12 @@
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>Earth attack for both sides UP</t>
+          <t>Earth Attack for all allies &amp; foes +25%</t>
         </is>
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7383,12 +7395,12 @@
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>Lightning attack for both sides UP</t>
+          <t>Lightning Attack for all allies &amp; foes +25%</t>
         </is>
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -7799,12 +7811,12 @@
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Less likely to trigger traps</t>
+          <t>Trap Trigger Rate -50%</t>
         </is>
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8087,7 +8099,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Chest Mimic Appearance Rate UP</t>
+          <t>Chest Mimic Appearance Rate +50%</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -8343,12 +8355,12 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>Song skill efficacy UP</t>
+          <t>Song Potency +20% (Carol/Chorale etc.)</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8375,12 +8387,12 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>Song skill efficacy MiniUP</t>
+          <t>Song Potency +10%</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8407,12 +8419,12 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>Dance skill efficacy UP</t>
+          <t>Dance Potency +20%</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8439,12 +8451,12 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>Dance skill efficacy UP</t>
+          <t>Dance Potency +10%</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8471,12 +8483,12 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Doll skill efficacy UP</t>
+          <t>Doll Potency +20%</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>
@@ -8503,12 +8515,12 @@
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>Doll skill efficacy MiniUP</t>
+          <t>Doll Potency +10%</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t>Vanilla</t>
+          <t>Approved</t>
         </is>
       </c>
     </row>

</xml_diff>